<commit_message>
Track the guide screenshot retake and the code review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46320.81182753472</v>
+        <v>46321.55850734954</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>38:46</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="H3" t="n">
-        <v>778</v>
+        <v>929</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>1546</v>
+        <v>1844</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>3483843</v>
+        <v>6049765</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>350124744</v>
+        <v>437510697</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1356481</v>
+        <v>1530179</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>354966614</v>
+        <v>445092485</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Tenant creation, reporter registry and NPI/CLIA import, extract findings and submit, operations and NPI/CLIA user guides, PR</t>
+          <t>Guide screenshots retaken (PR #5); code review with 16 issues filed (#6-#21)</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-25 19:29:03 (local time)</t>
+          <t>Last refreshed: 2026-10-26 13:24:31 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker T174-T178 and usage journal for issues #10, #11, #12, #15, #16
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46321.77317405093</v>
+        <v>46321.80967540509</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>43:55</t>
+          <t>44:47</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H3" t="n">
-        <v>1150</v>
+        <v>1199</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>2286</v>
+        <v>2384</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>6671596</v>
+        <v>6753022</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>530471028</v>
+        <v>549151577</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1738974</v>
+        <v>1786987</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>538883884</v>
+        <v>557693970</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Issue #29 task links and cross-tenant suite</t>
+          <t>Issues #10 #11 #12 #15 #16</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-26 18:33:30 (local time)</t>
+          <t>Last refreshed: 2026-10-26 19:26:09 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker T179-T182 and usage journal for issues #13, #17, #18, #19
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46321.80967540509</v>
+        <v>46321.82281681713</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>44:47</t>
+          <t>45:06</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H3" t="n">
-        <v>1199</v>
+        <v>1235</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>2384</v>
+        <v>2456</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>6753022</v>
+        <v>6822910</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>549151577</v>
+        <v>565557534</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1786987</v>
+        <v>1821380</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>557693970</v>
+        <v>574204280</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Issues #10 #11 #12 #15 #16</t>
+          <t>Issues #13 #17 #18 #19</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-26 19:26:09 (local time)</t>
+          <t>Last refreshed: 2026-10-26 19:45:06 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker T183-T185 and usage journal for issues #20, #21 and the guides
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46321.82281681713</v>
+        <v>46321.84793991898</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>45:06</t>
+          <t>45:42</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H3" t="n">
-        <v>1235</v>
+        <v>1310</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>2456</v>
+        <v>2604</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>6822910</v>
+        <v>6993775</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>565557534</v>
+        <v>608009643</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1821380</v>
+        <v>1887408</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>574204280</v>
+        <v>616893430</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Issues #13 #17 #18 #19</t>
+          <t>Issues #20 #21 and guide PDFs</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-26 19:45:06 (local time)</t>
+          <t>Last refreshed: 2026-10-26 20:21:05 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker T186 and usage journal for issue #26
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46321.84793991898</v>
+        <v>46321.85536850694</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>45:42</t>
+          <t>45:53</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H3" t="n">
-        <v>1310</v>
+        <v>1318</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>2604</v>
+        <v>2620</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>6993775</v>
+        <v>7003630</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>608009643</v>
+        <v>613347897</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1887408</v>
+        <v>1894286</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>616893430</v>
+        <v>622248433</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Issues #20 #21 and guide PDFs</t>
+          <t>Issue #26 profile version</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-26 20:21:05 (local time)</t>
+          <t>Last refreshed: 2026-10-26 20:32:00 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker and journal: UX review and the first batch of UX fixes
T187 records the UX review (issues #36 to #51); T188 to T195 record the fixes
for #36, #37/#38, #39, #40, #41, #43, #44 and #47.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46321.85536850694</v>
+        <v>46322.24387145833</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>45:53</t>
+          <t>55:13</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H3" t="n">
-        <v>1318</v>
+        <v>1488</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>2620</v>
+        <v>2958</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>7003630</v>
+        <v>9028768</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>613347897</v>
+        <v>726414961</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1894286</v>
+        <v>2059444</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>622248433</v>
+        <v>737506131</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Issue #26 profile version</t>
+          <t>UX review batch 1: issues #36 #37 #38 #39 #40 #41 #43 #44 #47 (time zones, display names, dates, held records on Home, bulk assign, status pages, first sign-in, phone layout)</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-26 20:32:00 (local time)</t>
+          <t>Last refreshed: 2026-10-27 05:51:13 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker and journal: UX fixes batch 2
T196 to T198 record the fixes for #46, #51 and #49.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>claude-opus-5-5</t>
+          <t>&lt;synthetic&gt;</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46322.24387145833</v>
+        <v>46322.36230244213</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>55:13</t>
+          <t>58:03</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" t="n">
-        <v>1488</v>
+        <v>1548</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>2958</v>
+        <v>3076</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>9028768</v>
+        <v>9240143</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>726414961</v>
+        <v>737214256</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>2059444</v>
+        <v>2119479</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>737506131</v>
+        <v>748576954</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>UX review batch 1: issues #36 #37 #38 #39 #40 #41 #43 #44 #47 (time zones, display names, dates, held records on Home, bulk assign, status pages, first sign-in, phone layout)</t>
+          <t>UX review batch 2: issues #46 #51 #49 (form errors, heading focus ring, timeline axis); logged #53 (CSP nonce encoding)</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-27 05:51:13 (local time)</t>
+          <t>Last refreshed: 2026-10-27 08:42:04 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker and journal: CSP nonce fix (#53)
T199 records the fix for #53.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>&lt;synthetic&gt;</t>
+          <t>claude-opus-5-5</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46322.36230244213</v>
+        <v>46322.38455262731</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>58:03</t>
+          <t>58:35</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H3" t="n">
-        <v>1548</v>
+        <v>1560</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>3076</v>
+        <v>3100</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>9240143</v>
+        <v>9253614</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>737214256</v>
+        <v>740145933</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>2119479</v>
+        <v>2127533</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>748576954</v>
+        <v>751530180</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>UX review batch 2: issues #46 #51 #49 (form errors, heading focus ring, timeline axis); logged #53 (CSP nonce encoding)</t>
+          <t>Issue #53: CSP nonce in base64url so htmx partials keep their attributes</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-27 08:42:04 (local time)</t>
+          <t>Last refreshed: 2026-10-27 09:13:56 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker and journal: held rows to Match review (#42), audit log (#45)
T200 and T201 record the fixes for #42 and #45.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46322.38455262731</v>
+        <v>46322.56933050926</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>58:35</t>
+          <t>63:01</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H3" t="n">
-        <v>1560</v>
+        <v>1614</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>3100</v>
+        <v>3206</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>9253614</v>
+        <v>9565902</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>740145933</v>
+        <v>755673305</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>2127533</v>
+        <v>2174400</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>751530180</v>
+        <v>767416813</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Issue #53: CSP nonce in base64url so htmx partials keep their attributes</t>
+          <t>Issues #42 #45: held rows to Match review; audit log filters, paging, words, links, CSV</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-27 09:13:56 (local time)</t>
+          <t>Last refreshed: 2026-10-27 13:40:09 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker and journal: map context layer (#48)
T202 records the fix for #48.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46322.56933050926</v>
+        <v>46322.64870592592</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>63:01</t>
+          <t>64:56</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H3" t="n">
-        <v>1614</v>
+        <v>1665</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>3206</v>
+        <v>3308</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>9565902</v>
+        <v>10023879</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>755673305</v>
+        <v>774922415</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>2174400</v>
+        <v>2220143</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>767416813</v>
+        <v>787169745</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Issues #42 #45: held rows to Match review; audit log filters, paging, words, links, CSV</t>
+          <t>Issue #48: map county outlines, small cluster map, linked cluster tasks</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-27 13:40:09 (local time)</t>
+          <t>Last refreshed: 2026-10-27 15:34:26 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker and journal: cases list filters (#50)
T203 records the fix for #50.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal/MERIT_ClaudeCode_Usage.xlsx
+++ b/journal/MERIT_ClaudeCode_Usage.xlsx
@@ -604,37 +604,37 @@
         <v>46319.94307898148</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46322.64870592592</v>
+        <v>46322.70667160879</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>64:56</t>
+          <t>66:19</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H3" t="n">
-        <v>1665</v>
+        <v>1685</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>3308</v>
+        <v>3348</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>10023879</v>
+        <v>10461004</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>774922415</v>
+        <v>783332210</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>2220143</v>
+        <v>2247844</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>787169745</v>
+        <v>796044406</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Issue #48: map county outlines, small cluster map, linked cluster tasks</t>
+          <t>Issue #50: cases list filters, search, sorting, one-click unassigned</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-27 15:34:26 (local time)</t>
+          <t>Last refreshed: 2026-10-27 16:57:53 (local time)</t>
         </is>
       </c>
     </row>

</xml_diff>